<commit_message>
Add June_Individual Assignment Session 4
</commit_message>
<xml_diff>
--- a/outputs/expense_summary_en.xlsx
+++ b/outputs/expense_summary_en.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,14 @@
       </c>
       <c r="B6" t="n">
         <v>62977000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>69236000</v>
       </c>
     </row>
   </sheetData>
@@ -512,7 +520,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52811000</v>
+        <v>62984000</v>
       </c>
     </row>
     <row r="3">
@@ -527,7 +535,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45955000</v>
+        <v>58935000</v>
       </c>
     </row>
     <row r="4">
@@ -542,13 +550,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42407000</v>
+        <v>53879000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -557,13 +565,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28687000</v>
+        <v>34902000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -572,7 +580,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>26886000</v>
+        <v>32519000</v>
       </c>
     </row>
     <row r="7">
@@ -587,7 +595,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24305000</v>
+        <v>28003000</v>
       </c>
     </row>
     <row r="8">
@@ -602,7 +610,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>18198000</v>
+        <v>19181000</v>
       </c>
     </row>
     <row r="9">
@@ -617,37 +625,37 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>13209000</v>
+        <v>17416000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12473000</v>
+        <v>16626000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8970000</v>
+        <v>13371000</v>
       </c>
     </row>
     <row r="12">
@@ -662,37 +670,37 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6758000</v>
+        <v>8141000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5520000</v>
+        <v>6162000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3780000</v>
+        <v>5930000</v>
       </c>
     </row>
     <row r="15">
@@ -707,7 +715,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3521000</v>
+        <v>4256000</v>
       </c>
     </row>
     <row r="16">
@@ -722,7 +730,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3485000</v>
+        <v>3839000</v>
       </c>
     </row>
     <row r="17">
@@ -737,7 +745,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2957000</v>
+        <v>3014000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>